<commit_message>
cartos + autres docs
</commit_message>
<xml_diff>
--- a/Data/Questionnaires/Questionnaires_SLAM_B.xlsx
+++ b/Data/Questionnaires/Questionnaires_SLAM_B.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\Questionnaires\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9C4433-3DF1-472B-837A-C1640F1A3556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345533FE-A4F5-4C4E-BCDC-F1973C6CDC18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3479,7 +3479,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:CX79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3886,7 +3885,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>782</v>
       </c>
@@ -4256,7 +4255,7 @@
       <c r="CW3" s="3"/>
       <c r="CX3" s="3"/>
     </row>
-    <row r="4" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>782</v>
       </c>
@@ -4442,7 +4441,7 @@
       <c r="CW4" s="3"/>
       <c r="CX4" s="3"/>
     </row>
-    <row r="5" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>784</v>
       </c>
@@ -4578,7 +4577,7 @@
       <c r="CW5" s="3"/>
       <c r="CX5" s="3"/>
     </row>
-    <row r="6" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>782</v>
       </c>
@@ -4770,7 +4769,7 @@
       <c r="CW6" s="3"/>
       <c r="CX6" s="3"/>
     </row>
-    <row r="7" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>782</v>
       </c>
@@ -4954,7 +4953,7 @@
       <c r="CW7" s="3"/>
       <c r="CX7" s="3"/>
     </row>
-    <row r="8" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>782</v>
       </c>
@@ -5140,7 +5139,7 @@
       <c r="CW8" s="3"/>
       <c r="CX8" s="3"/>
     </row>
-    <row r="9" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>784</v>
       </c>
@@ -5276,7 +5275,7 @@
       <c r="CW9" s="3"/>
       <c r="CX9" s="3"/>
     </row>
-    <row r="10" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>782</v>
       </c>
@@ -5466,7 +5465,7 @@
       <c r="CW10" s="3"/>
       <c r="CX10" s="3"/>
     </row>
-    <row r="11" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>782</v>
       </c>
@@ -5632,7 +5631,7 @@
       <c r="CW11" s="3"/>
       <c r="CX11" s="3"/>
     </row>
-    <row r="12" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>782</v>
       </c>
@@ -5798,7 +5797,7 @@
       <c r="CW12" s="3"/>
       <c r="CX12" s="3"/>
     </row>
-    <row r="13" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>784</v>
       </c>
@@ -5936,7 +5935,7 @@
       <c r="CW13" s="3"/>
       <c r="CX13" s="3"/>
     </row>
-    <row r="14" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>782</v>
       </c>
@@ -6126,7 +6125,7 @@
       <c r="CW14" s="3"/>
       <c r="CX14" s="3"/>
     </row>
-    <row r="15" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>782</v>
       </c>
@@ -6314,7 +6313,7 @@
       <c r="CW15" s="3"/>
       <c r="CX15" s="3"/>
     </row>
-    <row r="16" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>784</v>
       </c>
@@ -6452,7 +6451,7 @@
       <c r="CW16" s="3"/>
       <c r="CX16" s="3"/>
     </row>
-    <row r="17" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>782</v>
       </c>
@@ -6636,7 +6635,7 @@
       <c r="CW17" s="3"/>
       <c r="CX17" s="3"/>
     </row>
-    <row r="18" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>782</v>
       </c>
@@ -6816,7 +6815,7 @@
       <c r="CW18" s="3"/>
       <c r="CX18" s="3"/>
     </row>
-    <row r="19" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>782</v>
       </c>
@@ -6998,7 +6997,7 @@
       <c r="CW19" s="3"/>
       <c r="CX19" s="3"/>
     </row>
-    <row r="20" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>782</v>
       </c>
@@ -7188,7 +7187,7 @@
       <c r="CW20" s="3"/>
       <c r="CX20" s="3"/>
     </row>
-    <row r="21" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>782</v>
       </c>
@@ -7380,7 +7379,7 @@
       <c r="CW21" s="3"/>
       <c r="CX21" s="3"/>
     </row>
-    <row r="22" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>782</v>
       </c>
@@ -7558,7 +7557,7 @@
       <c r="CW22" s="3"/>
       <c r="CX22" s="3"/>
     </row>
-    <row r="23" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>782</v>
       </c>
@@ -7740,7 +7739,7 @@
       <c r="CW23" s="3"/>
       <c r="CX23" s="3"/>
     </row>
-    <row r="24" spans="1:102" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:102" ht="87" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>782</v>
       </c>
@@ -7922,7 +7921,7 @@
       <c r="CW24" s="3"/>
       <c r="CX24" s="3"/>
     </row>
-    <row r="25" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>782</v>
       </c>
@@ -8516,7 +8515,7 @@
       <c r="CW27" s="3"/>
       <c r="CX27" s="3"/>
     </row>
-    <row r="28" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>784</v>
       </c>
@@ -8652,7 +8651,7 @@
       <c r="CW28" s="3"/>
       <c r="CX28" s="3"/>
     </row>
-    <row r="29" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>782</v>
       </c>
@@ -9022,7 +9021,7 @@
       <c r="CW30" s="3"/>
       <c r="CX30" s="3"/>
     </row>
-    <row r="31" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>782</v>
       </c>
@@ -9206,7 +9205,7 @@
       <c r="CW31" s="3"/>
       <c r="CX31" s="3"/>
     </row>
-    <row r="32" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>782</v>
       </c>
@@ -9382,7 +9381,7 @@
       <c r="CW32" s="3"/>
       <c r="CX32" s="3"/>
     </row>
-    <row r="33" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>782</v>
       </c>
@@ -9580,7 +9579,7 @@
       <c r="CW33" s="3"/>
       <c r="CX33" s="3"/>
     </row>
-    <row r="34" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>784</v>
       </c>
@@ -9716,7 +9715,7 @@
       <c r="CW34" s="3"/>
       <c r="CX34" s="3"/>
     </row>
-    <row r="35" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>782</v>
       </c>
@@ -9900,7 +9899,7 @@
       <c r="CW35" s="3"/>
       <c r="CX35" s="3"/>
     </row>
-    <row r="36" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>782</v>
       </c>
@@ -10064,7 +10063,7 @@
       <c r="CW36" s="3"/>
       <c r="CX36" s="3"/>
     </row>
-    <row r="37" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>782</v>
       </c>
@@ -10252,7 +10251,7 @@
       <c r="CW37" s="3"/>
       <c r="CX37" s="3"/>
     </row>
-    <row r="38" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>783</v>
       </c>
@@ -10444,7 +10443,7 @@
       <c r="CW38" s="3"/>
       <c r="CX38" s="3"/>
     </row>
-    <row r="39" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>783</v>
       </c>
@@ -10632,7 +10631,7 @@
       <c r="CW39" s="3"/>
       <c r="CX39" s="3"/>
     </row>
-    <row r="40" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>783</v>
       </c>
@@ -10818,7 +10817,7 @@
       <c r="CW40" s="3"/>
       <c r="CX40" s="3"/>
     </row>
-    <row r="41" spans="1:102" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:102" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>783</v>
       </c>
@@ -11008,7 +11007,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="42" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>783</v>
       </c>
@@ -11196,7 +11195,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="43" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>783</v>
       </c>
@@ -11380,7 +11379,7 @@
       <c r="CW43" s="3"/>
       <c r="CX43" s="3"/>
     </row>
-    <row r="44" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>783</v>
       </c>
@@ -11576,7 +11575,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="45" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
         <v>783</v>
       </c>
@@ -11764,7 +11763,7 @@
       <c r="CW45" s="3"/>
       <c r="CX45" s="3"/>
     </row>
-    <row r="46" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>783</v>
       </c>
@@ -11954,7 +11953,7 @@
       <c r="CW46" s="3"/>
       <c r="CX46" s="3"/>
     </row>
-    <row r="47" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>783</v>
       </c>
@@ -12146,7 +12145,7 @@
       <c r="CW47" s="3"/>
       <c r="CX47" s="3"/>
     </row>
-    <row r="48" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>783</v>
       </c>
@@ -12332,7 +12331,7 @@
       <c r="CW48" s="3"/>
       <c r="CX48" s="3"/>
     </row>
-    <row r="49" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
         <v>784</v>
       </c>
@@ -12460,7 +12459,7 @@
       <c r="CW49" s="3"/>
       <c r="CX49" s="3"/>
     </row>
-    <row r="50" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>783</v>
       </c>
@@ -12646,7 +12645,7 @@
       <c r="CW50" s="3"/>
       <c r="CX50" s="3"/>
     </row>
-    <row r="51" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>783</v>
       </c>
@@ -12834,7 +12833,7 @@
       <c r="CW51" s="3"/>
       <c r="CX51" s="3"/>
     </row>
-    <row r="52" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
         <v>784</v>
       </c>
@@ -12958,7 +12957,7 @@
       <c r="CW52" s="3"/>
       <c r="CX52" s="3"/>
     </row>
-    <row r="53" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
         <v>784</v>
       </c>
@@ -13082,7 +13081,7 @@
       <c r="CW53" s="3"/>
       <c r="CX53" s="3"/>
     </row>
-    <row r="54" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>784</v>
       </c>
@@ -13206,7 +13205,7 @@
       <c r="CW54" s="3"/>
       <c r="CX54" s="3"/>
     </row>
-    <row r="55" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>784</v>
       </c>
@@ -13330,7 +13329,7 @@
       <c r="CW55" s="3"/>
       <c r="CX55" s="3"/>
     </row>
-    <row r="56" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>784</v>
       </c>
@@ -13454,7 +13453,7 @@
       <c r="CW56" s="3"/>
       <c r="CX56" s="3"/>
     </row>
-    <row r="57" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
         <v>784</v>
       </c>
@@ -13578,7 +13577,7 @@
       <c r="CW57" s="3"/>
       <c r="CX57" s="3"/>
     </row>
-    <row r="58" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>784</v>
       </c>
@@ -13702,7 +13701,7 @@
       <c r="CW58" s="3"/>
       <c r="CX58" s="3"/>
     </row>
-    <row r="59" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
         <v>784</v>
       </c>
@@ -13826,7 +13825,7 @@
       <c r="CW59" s="3"/>
       <c r="CX59" s="3"/>
     </row>
-    <row r="60" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>784</v>
       </c>
@@ -13950,7 +13949,7 @@
       <c r="CW60" s="3"/>
       <c r="CX60" s="3"/>
     </row>
-    <row r="61" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>784</v>
       </c>
@@ -14074,7 +14073,7 @@
       <c r="CW61" s="3"/>
       <c r="CX61" s="3"/>
     </row>
-    <row r="62" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>784</v>
       </c>
@@ -14198,7 +14197,7 @@
       <c r="CW62" s="3"/>
       <c r="CX62" s="3"/>
     </row>
-    <row r="63" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>784</v>
       </c>
@@ -14322,7 +14321,7 @@
       <c r="CW63" s="3"/>
       <c r="CX63" s="3"/>
     </row>
-    <row r="64" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>784</v>
       </c>
@@ -14446,7 +14445,7 @@
       <c r="CW64" s="3"/>
       <c r="CX64" s="3"/>
     </row>
-    <row r="65" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
         <v>784</v>
       </c>
@@ -14570,7 +14569,7 @@
       <c r="CW65" s="3"/>
       <c r="CX65" s="3"/>
     </row>
-    <row r="66" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
         <v>784</v>
       </c>
@@ -14694,7 +14693,7 @@
       <c r="CW66" s="3"/>
       <c r="CX66" s="3"/>
     </row>
-    <row r="67" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>784</v>
       </c>
@@ -14818,7 +14817,7 @@
       <c r="CW67" s="3"/>
       <c r="CX67" s="3"/>
     </row>
-    <row r="68" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
         <v>784</v>
       </c>
@@ -14942,7 +14941,7 @@
       <c r="CW68" s="3"/>
       <c r="CX68" s="3"/>
     </row>
-    <row r="69" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
         <v>784</v>
       </c>
@@ -15066,7 +15065,7 @@
       <c r="CW69" s="3"/>
       <c r="CX69" s="3"/>
     </row>
-    <row r="70" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
         <v>784</v>
       </c>
@@ -15190,7 +15189,7 @@
       <c r="CW70" s="3"/>
       <c r="CX70" s="3"/>
     </row>
-    <row r="71" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
         <v>784</v>
       </c>
@@ -15314,7 +15313,7 @@
       <c r="CW71" s="3"/>
       <c r="CX71" s="3"/>
     </row>
-    <row r="72" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>784</v>
       </c>
@@ -15438,7 +15437,7 @@
       <c r="CW72" s="3"/>
       <c r="CX72" s="3"/>
     </row>
-    <row r="73" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
         <v>784</v>
       </c>
@@ -15562,7 +15561,7 @@
       <c r="CW73" s="3"/>
       <c r="CX73" s="3"/>
     </row>
-    <row r="74" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>784</v>
       </c>
@@ -15686,7 +15685,7 @@
       <c r="CW74" s="3"/>
       <c r="CX74" s="3"/>
     </row>
-    <row r="75" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>784</v>
       </c>
@@ -15810,7 +15809,7 @@
       <c r="CW75" s="3"/>
       <c r="CX75" s="3"/>
     </row>
-    <row r="76" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
         <v>784</v>
       </c>
@@ -15934,7 +15933,7 @@
       <c r="CW76" s="3"/>
       <c r="CX76" s="3"/>
     </row>
-    <row r="77" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
         <v>784</v>
       </c>
@@ -16058,7 +16057,7 @@
       <c r="CW77" s="3"/>
       <c r="CX77" s="3"/>
     </row>
-    <row r="78" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
         <v>784</v>
       </c>
@@ -16182,7 +16181,7 @@
       <c r="CW78" s="3"/>
       <c r="CX78" s="3"/>
     </row>
-    <row r="79" spans="1:102" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>784</v>
       </c>
@@ -16307,29 +16306,7 @@
       <c r="CX79" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CX79" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="CODES"/>
-        <filter val="DATA"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="7">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="8">
-      <filters>
-        <filter val="1.4b"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="10">
-      <filters>
-        <filter val="PRODUITES"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:CX79" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="D38" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="S14" r:id="rId2" xr:uid="{6EAA74DF-1F24-4AAC-B3D4-3D02BD34995E}"/>

</xml_diff>